<commit_message>
Redesign reasoning page, fix local API detection, speed up /health endpoint
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/0602_service-offerings-catalog_reviewed.xlsx
+++ b/docs/0602_service-offerings-catalog_reviewed.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmc365-my.sharepoint.com/personal/h-ono_cmc_co_jp/Documents/デスクトップ/次世代商談/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="18" documentId="13_ncr:1_{55198819-8B1B-44B6-99A0-B0A0D0078AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{8B6D1D81-3D15-44AC-A439-C160CDCB56E5}"/>
+  <xr:revisionPtr revIDLastSave="24" documentId="13_ncr:1_{55198819-8B1B-44B6-99A0-B0A0D0078AB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA080780-021A-4E71-92E2-59280CC767E6}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="記入" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="537">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1100" uniqueCount="539">
   <si>
     <t>id</t>
   </si>
@@ -1669,6 +1669,14 @@
   </si>
   <si>
     <t>SOSボタンの取り外し</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>情報過多による判断負荷</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>機能不足による後悔</t>
     <phoneticPr fontId="2"/>
   </si>
 </sst>
@@ -2890,7 +2898,7 @@
         <v>329</v>
       </c>
       <c r="M14" s="14" t="s">
-        <v>331</v>
+        <v>537</v>
       </c>
       <c r="N14" s="14" t="s">
         <v>54</v>
@@ -3520,7 +3528,7 @@
         <v>331</v>
       </c>
       <c r="M24" s="14" t="s">
-        <v>333</v>
+        <v>538</v>
       </c>
       <c r="N24" s="14" t="s">
         <v>54</v>

</xml_diff>